<commit_message>
chore(data): sync latest auction results for 2026-09-22 16:16
</commit_message>
<xml_diff>
--- a/data/蒙煤拍卖临时记录.xlsx
+++ b/data/蒙煤拍卖临时记录.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -3245,7 +3245,9 @@
       <c r="G49" s="10" t="n">
         <v>181.5</v>
       </c>
-      <c r="H49" s="10" t="n"/>
+      <c r="H49" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="I49" s="15">
         <f>(H49-G49)/G49</f>
         <v/>

</xml_diff>

<commit_message>
fix: remove ghost notice duplicate records, add port tags to chart dates and location tooltips
</commit_message>
<xml_diff>
--- a/data/蒙煤拍卖临时记录.xlsx
+++ b/data/蒙煤拍卖临时记录.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
feat(sync): exclude Fe-65% products, clean database records and update datasets
</commit_message>
<xml_diff>
--- a/data/蒙煤拍卖临时记录.xlsx
+++ b/data/蒙煤拍卖临时记录.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,9 +17,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -66,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -77,19 +77,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -457,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -552,7 +546,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D2" s="7" t="n">
+      <c r="D2" s="4" t="n">
         <v>46261.41666666666</v>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -571,7 +565,7 @@
       <c r="H2" s="2" t="n">
         <v>1340</v>
       </c>
-      <c r="I2" s="8">
+      <c r="I2" s="5">
         <f>(H2-G2)/G2</f>
         <v/>
       </c>
@@ -608,7 +602,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D3" s="7" t="n">
+      <c r="D3" s="4" t="n">
         <v>46261.41666666666</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -627,7 +621,7 @@
       <c r="H3" s="6" t="n">
         <v>190.5</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="5">
         <f>(H3-G3)/G3</f>
         <v/>
       </c>
@@ -663,7 +657,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D4" s="7" t="n">
+      <c r="D4" s="4" t="n">
         <v>46262.41666666666</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -682,7 +676,7 @@
       <c r="H4" s="2" t="n">
         <v>1405</v>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="5">
         <f>(H4-G4)/G4</f>
         <v/>
       </c>
@@ -719,7 +713,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="4" t="n">
         <v>46262.41666666666</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -738,7 +732,7 @@
       <c r="H5" s="6" t="n">
         <v>198.5</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="5">
         <f>(H5-G5)/G5</f>
         <v/>
       </c>
@@ -774,7 +768,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="4" t="n">
         <v>46262.5</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -793,7 +787,7 @@
       <c r="H6" s="6" t="n">
         <v>194.5</v>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="5">
         <f>(H6-G6)/G6</f>
         <v/>
       </c>
@@ -829,7 +823,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="4" t="n">
         <v>46265.41666666666</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -848,7 +842,7 @@
       <c r="H7" s="2" t="n">
         <v>1515</v>
       </c>
-      <c r="I7" s="8">
+      <c r="I7" s="5">
         <f>(H7-G7)/G7</f>
         <v/>
       </c>
@@ -885,7 +879,7 @@
           <t>坎加德勘探 有限责任公司</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="4" t="n">
         <v>46266.41666666666</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -904,7 +898,7 @@
       <c r="H8" s="2" t="n">
         <v>1205</v>
       </c>
-      <c r="I8" s="8">
+      <c r="I8" s="5">
         <f>(H8-G8)/G8</f>
         <v/>
       </c>
@@ -941,7 +935,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="4" t="n">
         <v>46267.41666666666</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -960,7 +954,7 @@
       <c r="H9" s="2" t="n">
         <v>1405</v>
       </c>
-      <c r="I9" s="8">
+      <c r="I9" s="5">
         <f>(H9-G9)/G9</f>
         <v/>
       </c>
@@ -997,7 +991,7 @@
           <t>塔万陶勒盖股份公司</t>
         </is>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="4" t="n">
         <v>46267.45833333334</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -1016,7 +1010,7 @@
       <c r="H10" s="6" t="n">
         <v>211.5</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="5">
         <f>(H10-G10)/G10</f>
         <v/>
       </c>
@@ -1052,7 +1046,7 @@
           <t>塔万陶勒盖股份公司</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="4" t="n">
         <v>46267.58333333334</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1071,7 +1065,7 @@
       <c r="H11" s="6" t="n">
         <v>212.5</v>
       </c>
-      <c r="I11" s="8">
+      <c r="I11" s="5">
         <f>(H11-G11)/G11</f>
         <v/>
       </c>
@@ -1107,7 +1101,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="4" t="n">
         <v>46268.41666666666</v>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1126,7 +1120,7 @@
       <c r="H12" s="6" t="n">
         <v>171.4</v>
       </c>
-      <c r="I12" s="8">
+      <c r="I12" s="5">
         <f>(H12-G12)/G12</f>
         <v/>
       </c>
@@ -1163,7 +1157,7 @@
           <t>塔万陶勒盖股份公司</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="4" t="n">
         <v>46269.41666666666</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1182,7 +1176,7 @@
       <c r="H13" s="6" t="n">
         <v>210.5</v>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="5">
         <f>(H13-G13)/G13</f>
         <v/>
       </c>
@@ -1218,7 +1212,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="4" t="n">
         <v>46269.41666666666</v>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1237,7 +1231,7 @@
       <c r="H14" s="2" t="n">
         <v>188</v>
       </c>
-      <c r="I14" s="8">
+      <c r="I14" s="5">
         <f>(H14-G14)/G14</f>
         <v/>
       </c>
@@ -1274,7 +1268,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="4" t="n">
         <v>46269.41666666666</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1293,7 +1287,7 @@
       <c r="H15" s="2" t="n">
         <v>1445</v>
       </c>
-      <c r="I15" s="8">
+      <c r="I15" s="5">
         <f>(H15-G15)/G15</f>
         <v/>
       </c>
@@ -1330,7 +1324,7 @@
           <t>塔万陶勒盖股份公司</t>
         </is>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="4" t="n">
         <v>46269.58333333334</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1349,7 +1343,7 @@
       <c r="H16" s="6" t="n">
         <v>208.5</v>
       </c>
-      <c r="I16" s="8">
+      <c r="I16" s="5">
         <f>(H16-G16)/G16</f>
         <v/>
       </c>
@@ -1385,7 +1379,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="4" t="n">
         <v>46272.41666666666</v>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1404,7 +1398,7 @@
       <c r="H17" s="2" t="n">
         <v>197</v>
       </c>
-      <c r="I17" s="8">
+      <c r="I17" s="5">
         <f>(H17-G17)/G17</f>
         <v/>
       </c>
@@ -1441,7 +1435,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="D18" s="4" t="n">
         <v>46272.41666666666</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1460,7 +1454,7 @@
       <c r="H18" s="2" t="n">
         <v>1455</v>
       </c>
-      <c r="I18" s="8">
+      <c r="I18" s="5">
         <f>(H18-G18)/G18</f>
         <v/>
       </c>
@@ -1497,7 +1491,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D19" s="4" t="n">
         <v>46272.5</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1516,7 +1510,7 @@
       <c r="H19" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I19" s="8">
+      <c r="I19" s="5">
         <f>(H19-G19)/G19</f>
         <v/>
       </c>
@@ -1553,7 +1547,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D20" s="7" t="n">
+      <c r="D20" s="4" t="n">
         <v>46273.41666666666</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1572,7 +1566,7 @@
       <c r="H20" s="6" t="n">
         <v>193.5</v>
       </c>
-      <c r="I20" s="8">
+      <c r="I20" s="5">
         <f>(H20-G20)/G20</f>
         <v/>
       </c>
@@ -1609,7 +1603,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="D21" s="4" t="n">
         <v>46274.41666666666</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1628,7 +1622,7 @@
       <c r="H21" s="2" t="n">
         <v>192</v>
       </c>
-      <c r="I21" s="8">
+      <c r="I21" s="5">
         <f>(H21-G21)/G21</f>
         <v/>
       </c>
@@ -1665,7 +1659,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D22" s="7" t="n">
+      <c r="D22" s="4" t="n">
         <v>46274.41666666666</v>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -1684,7 +1678,7 @@
       <c r="H22" s="2" t="n">
         <v>1435</v>
       </c>
-      <c r="I22" s="8">
+      <c r="I22" s="5">
         <f>(H22-G22)/G22</f>
         <v/>
       </c>
@@ -1721,7 +1715,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D23" s="7" t="n">
+      <c r="D23" s="4" t="n">
         <v>46274.66666666666</v>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1740,7 +1734,7 @@
       <c r="H23" s="6" t="n">
         <v>187.5</v>
       </c>
-      <c r="I23" s="8">
+      <c r="I23" s="5">
         <f>(H23-G23)/G23</f>
         <v/>
       </c>
@@ -1777,7 +1771,7 @@
           <t>塔万陶勒盖股份公司</t>
         </is>
       </c>
-      <c r="D24" s="7" t="n">
+      <c r="D24" s="4" t="n">
         <v>46275.45833333334</v>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1796,7 +1790,7 @@
       <c r="H24" s="6" t="n">
         <v>120.5</v>
       </c>
-      <c r="I24" s="8">
+      <c r="I24" s="5">
         <f>(H24-G24)/G24</f>
         <v/>
       </c>
@@ -1832,7 +1826,7 @@
           <t>塔万陶勒盖股份公司</t>
         </is>
       </c>
-      <c r="D25" s="7" t="n">
+      <c r="D25" s="4" t="n">
         <v>46276.41666666666</v>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1851,7 +1845,7 @@
       <c r="H25" s="2" t="n">
         <v>191</v>
       </c>
-      <c r="I25" s="8">
+      <c r="I25" s="5">
         <f>(H25-G25)/G25</f>
         <v/>
       </c>
@@ -1887,7 +1881,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D26" s="7" t="n">
+      <c r="D26" s="4" t="n">
         <v>46276.41666666666</v>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1906,7 +1900,7 @@
       <c r="H26" s="2" t="n">
         <v>1445</v>
       </c>
-      <c r="I26" s="8">
+      <c r="I26" s="5">
         <f>(H26-G26)/G26</f>
         <v/>
       </c>
@@ -1942,7 +1936,7 @@
           <t>塔万陶勒盖股份公司</t>
         </is>
       </c>
-      <c r="D27" s="7" t="n">
+      <c r="D27" s="4" t="n">
         <v>46276.45833333334</v>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1961,7 +1955,7 @@
       <c r="H27" s="2" t="n">
         <v>191</v>
       </c>
-      <c r="I27" s="8">
+      <c r="I27" s="5">
         <f>(H27-G27)/G27</f>
         <v/>
       </c>
@@ -1997,7 +1991,7 @@
           <t>塔万陶勒盖股份公司</t>
         </is>
       </c>
-      <c r="D28" s="7" t="n">
+      <c r="D28" s="4" t="n">
         <v>46276.58333333334</v>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -2016,7 +2010,7 @@
       <c r="H28" s="2" t="n">
         <v>160</v>
       </c>
-      <c r="I28" s="8">
+      <c r="I28" s="5">
         <f>(H28-G28)/G28</f>
         <v/>
       </c>
@@ -2052,7 +2046,7 @@
           <t>塔万陶勒盖股份公司</t>
         </is>
       </c>
-      <c r="D29" s="7" t="n">
+      <c r="D29" s="4" t="n">
         <v>46276.625</v>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -2071,7 +2065,7 @@
       <c r="H29" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I29" s="8">
+      <c r="I29" s="5">
         <f>(H29-G29)/G29</f>
         <v/>
       </c>
@@ -2107,7 +2101,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D30" s="7" t="n">
+      <c r="D30" s="4" t="n">
         <v>46279.41666666666</v>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -2126,7 +2120,7 @@
       <c r="H30" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I30" s="8">
+      <c r="I30" s="5">
         <f>(H30-G30)/G30</f>
         <v/>
       </c>
@@ -2162,7 +2156,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D31" s="7" t="n">
+      <c r="D31" s="4" t="n">
         <v>46279.41666666666</v>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -2181,7 +2175,7 @@
       <c r="H31" s="2" t="n">
         <v>1420</v>
       </c>
-      <c r="I31" s="8">
+      <c r="I31" s="5">
         <f>(H31-G31)/G31</f>
         <v/>
       </c>
@@ -2217,7 +2211,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D32" s="7" t="n">
+      <c r="D32" s="4" t="n">
         <v>46279.45833333334</v>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -2236,7 +2230,7 @@
       <c r="H32" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I32" s="8">
+      <c r="I32" s="5">
         <f>(H32-G32)/G32</f>
         <v/>
       </c>
@@ -2272,7 +2266,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D33" s="7" t="n">
+      <c r="D33" s="4" t="n">
         <v>46279.58333333334</v>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -2291,7 +2285,7 @@
       <c r="H33" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I33" s="8">
+      <c r="I33" s="5">
         <f>(H33-G33)/G33</f>
         <v/>
       </c>
@@ -2327,7 +2321,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D34" s="7" t="n">
+      <c r="D34" s="4" t="n">
         <v>46279.625</v>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2346,7 +2340,7 @@
       <c r="H34" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I34" s="8">
+      <c r="I34" s="5">
         <f>(H34-G34)/G34</f>
         <v/>
       </c>
@@ -2382,7 +2376,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D35" s="7" t="n">
+      <c r="D35" s="4" t="n">
         <v>46280.41666666666</v>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -2401,7 +2395,7 @@
       <c r="H35" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I35" s="8">
+      <c r="I35" s="5">
         <f>(H35-G35)/G35</f>
         <v/>
       </c>
@@ -2437,7 +2431,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D36" s="7" t="n">
+      <c r="D36" s="4" t="n">
         <v>46280.58333333334</v>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2456,7 +2450,7 @@
       <c r="H36" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I36" s="8">
+      <c r="I36" s="5">
         <f>(H36-G36)/G36</f>
         <v/>
       </c>
@@ -2492,7 +2486,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D37" s="7" t="n">
+      <c r="D37" s="4" t="n">
         <v>46281.41666666666</v>
       </c>
       <c r="E37" s="3" t="inlineStr">
@@ -2511,7 +2505,7 @@
       <c r="H37" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I37" s="8">
+      <c r="I37" s="5">
         <f>(H37-G37)/G37</f>
         <v/>
       </c>
@@ -2547,7 +2541,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D38" s="7" t="n">
+      <c r="D38" s="4" t="n">
         <v>46281.41666666666</v>
       </c>
       <c r="E38" s="3" t="inlineStr">
@@ -2566,7 +2560,7 @@
       <c r="H38" s="2" t="n">
         <v>1405</v>
       </c>
-      <c r="I38" s="8">
+      <c r="I38" s="5">
         <f>(H38-G38)/G38</f>
         <v/>
       </c>
@@ -2602,7 +2596,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D39" s="7" t="n">
+      <c r="D39" s="4" t="n">
         <v>46281.58333333334</v>
       </c>
       <c r="E39" s="3" t="inlineStr">
@@ -2621,7 +2615,7 @@
       <c r="H39" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I39" s="8">
+      <c r="I39" s="5">
         <f>(H39-G39)/G39</f>
         <v/>
       </c>
@@ -2657,7 +2651,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D40" s="7" t="n">
+      <c r="D40" s="4" t="n">
         <v>46282.41666666666</v>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2676,7 +2670,7 @@
       <c r="H40" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I40" s="8">
+      <c r="I40" s="5">
         <f>(H40-G40)/G40</f>
         <v/>
       </c>
@@ -2712,7 +2706,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D41" s="7" t="n">
+      <c r="D41" s="4" t="n">
         <v>46282.58333333334</v>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -2731,7 +2725,7 @@
       <c r="H41" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I41" s="8">
+      <c r="I41" s="5">
         <f>(H41-G41)/G41</f>
         <v/>
       </c>
@@ -2767,7 +2761,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D42" s="7" t="n">
+      <c r="D42" s="4" t="n">
         <v>46283.41666666666</v>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2786,7 +2780,7 @@
       <c r="H42" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I42" s="8">
+      <c r="I42" s="5">
         <f>(H42-G42)/G42</f>
         <v/>
       </c>
@@ -2822,7 +2816,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D43" s="7" t="n">
+      <c r="D43" s="4" t="n">
         <v>46283.41666666666</v>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -2841,7 +2835,7 @@
       <c r="H43" s="2" t="n">
         <v>1255</v>
       </c>
-      <c r="I43" s="8">
+      <c r="I43" s="5">
         <f>(H43-G43)/G43</f>
         <v/>
       </c>
@@ -2877,7 +2871,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D44" s="7" t="n">
+      <c r="D44" s="4" t="n">
         <v>46283.58333333334</v>
       </c>
       <c r="E44" s="3" t="inlineStr">
@@ -2896,7 +2890,7 @@
       <c r="H44" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I44" s="8">
+      <c r="I44" s="5">
         <f>(H44-G44)/G44</f>
         <v/>
       </c>
@@ -2932,7 +2926,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D45" s="7" t="n">
+      <c r="D45" s="4" t="n">
         <v>46286.41666666666</v>
       </c>
       <c r="E45" s="3" t="inlineStr">
@@ -2951,7 +2945,7 @@
       <c r="H45" s="2" t="n">
         <v>1295</v>
       </c>
-      <c r="I45" s="8">
+      <c r="I45" s="5">
         <f>(H45-G45)/G45</f>
         <v/>
       </c>
@@ -2987,7 +2981,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D46" s="7" t="n">
+      <c r="D46" s="4" t="n">
         <v>46286.41666666666</v>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -3006,7 +3000,7 @@
       <c r="H46" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I46" s="8">
+      <c r="I46" s="5">
         <f>(H46-G46)/G46</f>
         <v/>
       </c>
@@ -3042,7 +3036,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D47" s="7" t="n">
+      <c r="D47" s="4" t="n">
         <v>46286.58333333334</v>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -3061,7 +3055,7 @@
       <c r="H47" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I47" s="8">
+      <c r="I47" s="5">
         <f>(H47-G47)/G47</f>
         <v/>
       </c>
@@ -3097,7 +3091,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D48" s="7" t="n">
+      <c r="D48" s="4" t="n">
         <v>46287.41666666666</v>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -3116,7 +3110,7 @@
       <c r="H48" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I48" s="8">
+      <c r="I48" s="5">
         <f>(H48-G48)/G48</f>
         <v/>
       </c>
@@ -3152,7 +3146,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D49" s="7" t="n">
+      <c r="D49" s="4" t="n">
         <v>46287.58333333334</v>
       </c>
       <c r="E49" s="3" t="inlineStr">
@@ -3171,7 +3165,7 @@
       <c r="H49" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I49" s="8">
+      <c r="I49" s="5">
         <f>(H49-G49)/G49</f>
         <v/>
       </c>
@@ -3207,7 +3201,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D50" s="7" t="n">
+      <c r="D50" s="4" t="n">
         <v>46288.41666666666</v>
       </c>
       <c r="E50" s="3" t="inlineStr">
@@ -3226,7 +3220,7 @@
       <c r="H50" s="2" t="n">
         <v>1290</v>
       </c>
-      <c r="I50" s="8">
+      <c r="I50" s="5">
         <f>(H50-G50)/G50</f>
         <v/>
       </c>
@@ -3262,7 +3256,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D51" s="7" t="n">
+      <c r="D51" s="4" t="n">
         <v>46288.41666666666</v>
       </c>
       <c r="E51" s="3" t="inlineStr">
@@ -3281,7 +3275,7 @@
       <c r="H51" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I51" s="8">
+      <c r="I51" s="5">
         <f>(H51-G51)/G51</f>
         <v/>
       </c>
@@ -3317,7 +3311,7 @@
           <t>埃尔登内斯·塔万陶勒盖有限责任公司</t>
         </is>
       </c>
-      <c r="D52" s="7" t="n">
+      <c r="D52" s="4" t="n">
         <v>46288.58333333334</v>
       </c>
       <c r="E52" s="3" t="inlineStr">
@@ -3336,7 +3330,7 @@
       <c r="H52" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I52" s="8">
+      <c r="I52" s="5">
         <f>(H52-G52)/G52</f>
         <v/>
       </c>
@@ -3372,7 +3366,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D53" s="7" t="n">
+      <c r="D53" s="4" t="n">
         <v>46290.41666666666</v>
       </c>
       <c r="E53" s="3" t="inlineStr">
@@ -3391,7 +3385,7 @@
       <c r="H53" s="2" t="n">
         <v>1285</v>
       </c>
-      <c r="I53" s="8">
+      <c r="I53" s="5">
         <f>(H53-G53)/G53</f>
         <v/>
       </c>
@@ -3427,7 +3421,7 @@
           <t>额尔登特矿业公司国资企业</t>
         </is>
       </c>
-      <c r="D54" s="7" t="n">
+      <c r="D54" s="4" t="n">
         <v>46290.625</v>
       </c>
       <c r="E54" s="3" t="inlineStr">
@@ -3440,13 +3434,13 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="G54" s="2" t="n">
+      <c r="G54" s="6" t="n">
         <v>3318.59</v>
       </c>
-      <c r="H54" s="2" t="n">
+      <c r="H54" s="6" t="n">
         <v>3613.59</v>
       </c>
-      <c r="I54" s="8">
+      <c r="I54" s="5">
         <f>(H54-G54)/G54</f>
         <v/>
       </c>
@@ -3482,7 +3476,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D55" s="7" t="n">
+      <c r="D55" s="4" t="n">
         <v>46293.41666666666</v>
       </c>
       <c r="E55" s="3" t="inlineStr">
@@ -3501,7 +3495,7 @@
       <c r="H55" s="2" t="n">
         <v>1260</v>
       </c>
-      <c r="I55" s="8">
+      <c r="I55" s="5">
         <f>(H55-G55)/G55</f>
         <v/>
       </c>
@@ -3537,7 +3531,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D56" s="7" t="n">
+      <c r="D56" s="4" t="n">
         <v>46295.41666666666</v>
       </c>
       <c r="E56" s="3" t="inlineStr">
@@ -3556,7 +3550,7 @@
       <c r="H56" s="2" t="n">
         <v>1265</v>
       </c>
-      <c r="I56" s="8">
+      <c r="I56" s="5">
         <f>(H56-G56)/G56</f>
         <v/>
       </c>
@@ -3592,7 +3586,7 @@
           <t>坎加德勘探 有限责任公司</t>
         </is>
       </c>
-      <c r="D57" s="7" t="n">
+      <c r="D57" s="4" t="n">
         <v>46296.58333333334</v>
       </c>
       <c r="E57" s="3" t="inlineStr">
@@ -3611,7 +3605,7 @@
       <c r="H57" s="2" t="n">
         <v>540</v>
       </c>
-      <c r="I57" s="8">
+      <c r="I57" s="5">
         <f>(H57-G57)/G57</f>
         <v/>
       </c>
@@ -3647,7 +3641,7 @@
           <t>塔万陶勒盖股份公司</t>
         </is>
       </c>
-      <c r="D58" s="7" t="n">
+      <c r="D58" s="4" t="n">
         <v>46297.41666666666</v>
       </c>
       <c r="E58" s="3" t="inlineStr">
@@ -3666,7 +3660,7 @@
       <c r="H58" s="2" t="n">
         <v>121</v>
       </c>
-      <c r="I58" s="8">
+      <c r="I58" s="5">
         <f>(H58-G58)/G58</f>
         <v/>
       </c>
@@ -3702,7 +3696,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D59" s="7" t="n">
+      <c r="D59" s="4" t="n">
         <v>46297.41666666666</v>
       </c>
       <c r="E59" s="3" t="inlineStr">
@@ -3721,7 +3715,7 @@
       <c r="H59" s="2" t="n">
         <v>1265</v>
       </c>
-      <c r="I59" s="8">
+      <c r="I59" s="5">
         <f>(H59-G59)/G59</f>
         <v/>
       </c>
@@ -3757,7 +3751,7 @@
           <t>能源资源有限责任公司</t>
         </is>
       </c>
-      <c r="D60" s="7" t="n">
+      <c r="D60" s="4" t="n">
         <v>46300.41666666666</v>
       </c>
       <c r="E60" s="3" t="inlineStr">
@@ -3774,7 +3768,7 @@
         <v>1150</v>
       </c>
       <c r="H60" s="2" t="n"/>
-      <c r="I60" s="8">
+      <c r="I60" s="5">
         <f>(H60-G60)/G60</f>
         <v/>
       </c>
@@ -3810,7 +3804,7 @@
           <t>塔万陶勒盖股份公司</t>
         </is>
       </c>
-      <c r="D61" s="7" t="n">
+      <c r="D61" s="4" t="n">
         <v>46301.41666666666</v>
       </c>
       <c r="E61" s="3" t="inlineStr">
@@ -3829,7 +3823,7 @@
       <c r="H61" s="2" t="n">
         <v>153</v>
       </c>
-      <c r="I61" s="8">
+      <c r="I61" s="5">
         <f>(H61-G61)/G61</f>
         <v/>
       </c>
@@ -3852,163 +3846,55 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>铁</t>
+          <t>煤炭</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Fe-65%</t>
+          <t>洗精主焦煤</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Mongolrostsvetmet SOE /Erdenes Critical Minerals SOE/</t>
-        </is>
-      </c>
-      <c r="D62" s="7" t="n">
-        <v>46301.45833333334</v>
+          <t>能源资源有限责任公司</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="n">
+        <v>46302.41666666666</v>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>1 批量/3300吨/</t>
+          <t>2 批量/12800吨/</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CNY</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>85</v>
+        <v>1150</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="I62" s="8">
+        <v>1250</v>
+      </c>
+      <c r="I62" s="5">
         <f>(H62-G62)/G62</f>
         <v/>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>2027年10月</t>
+          <t>2027年2月04日（最后供货日） DAP甘其毛都口岸</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>二连浩特铁路站</t>
+          <t>买方指定的甘其毛都口岸海关监管区</t>
         </is>
       </c>
       <c r="L62" s="3" t="inlineStr">
         <is>
-          <t>铁路</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>煤炭</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>洗精主焦煤</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>能源资源有限责任公司</t>
-        </is>
-      </c>
-      <c r="D63" s="7" t="n">
-        <v>46302.41666666666</v>
-      </c>
-      <c r="E63" s="3" t="inlineStr">
-        <is>
-          <t>2 批量/12800吨/</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="n">
-        <v>1150</v>
-      </c>
-      <c r="H63" s="2" t="n">
-        <v>1250</v>
-      </c>
-      <c r="I63" s="8">
-        <f>(H63-G63)/G63</f>
-        <v/>
-      </c>
-      <c r="J63" s="3" t="inlineStr">
-        <is>
-          <t>2027年2月04日（最后供货日） DAP甘其毛都口岸</t>
-        </is>
-      </c>
-      <c r="K63" s="3" t="inlineStr">
-        <is>
-          <t>买方指定的甘其毛都口岸海关监管区</t>
-        </is>
-      </c>
-      <c r="L63" s="3" t="inlineStr">
-        <is>
           <t>公路运输</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>铁</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>Fe-65%</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>Mongolrostsvetmet SOE /Erdenes Critical Minerals SOE/</t>
-        </is>
-      </c>
-      <c r="D64" s="7" t="n">
-        <v>46303.45833333334</v>
-      </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>1 批量/3300吨/</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="H64" s="2" t="n"/>
-      <c r="I64" s="8">
-        <f>(H64-G64)/G64</f>
-        <v/>
-      </c>
-      <c r="J64" s="3" t="inlineStr">
-        <is>
-          <t>2027年10月</t>
-        </is>
-      </c>
-      <c r="K64" s="3" t="inlineStr">
-        <is>
-          <t>二连浩特铁路站</t>
-        </is>
-      </c>
-      <c r="L64" s="3" t="inlineStr">
-        <is>
-          <t>铁路</t>
         </is>
       </c>
     </row>

</xml_diff>